<commit_message>
Add peer pharma PDF exports
</commit_message>
<xml_diff>
--- a/Merck Official Hackathon Corpus/manifest.xlsx
+++ b/Merck Official Hackathon Corpus/manifest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R6d34eed219af4659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R884b4b3bcbdb44b8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,10 +131,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifestTable" displayName="ManifestTable" ref="A1:P428" headerRowCount="1">
-  <x:autoFilter ref="A1:P428"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifestTable" displayName="ManifestTable" ref="A1:P444" headerRowCount="1">
+  <x:autoFilter ref="A1:P444"/>
   <x:tableColumns count="16">
-    <x:tableColumn id="1" name="﻿id"/>
+    <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="repository"/>
     <x:tableColumn id="3" name="subfolder"/>
     <x:tableColumn id="4" name="title"/>
@@ -213,12 +213,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -324,7 +370,7 @@
   <x:sheetData>
     <x:row r="1" ht="31.5" customHeight="1">
       <x:c r="A1" s="14" t="str">
-        <x:v>﻿id</x:v>
+        <x:v>id</x:v>
       </x:c>
       <x:c r="B1" s="14" t="str">
         <x:v>repository</x:v>
@@ -21080,15 +21126,719 @@
         <x:v>downloaded</x:v>
       </x:c>
     </x:row>
+    <x:row r="429">
+      <x:c r="A429" s="6" t="str">
+        <x:v>peerpdf-0001</x:v>
+      </x:c>
+      <x:c r="B429" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C429" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D429" s="6" t="str">
+        <x:v>Johnson &amp; Johnson 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E429" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F429" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G429" s="6" t="str"/>
+      <x:c r="H429" s="6" t="str"/>
+      <x:c r="I429" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=200406</x:v>
+      </x:c>
+      <x:c r="J429" s="6" t="str"/>
+      <x:c r="K429" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank01_johnson-and-johnson_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L429" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M429" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N429" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O429" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank01_johnson-and-johnson_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P429" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="430">
+      <x:c r="A430" s="6" t="str">
+        <x:v>peerpdf-0002</x:v>
+      </x:c>
+      <x:c r="B430" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C430" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D430" s="6" t="str">
+        <x:v>Roche Annual Report 2025 PDF export</x:v>
+      </x:c>
+      <x:c r="E430" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F430" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G430" s="6" t="str"/>
+      <x:c r="H430" s="6" t="str"/>
+      <x:c r="I430" s="6" t="str">
+        <x:v>https://www.roche.com/investors/annualreport25</x:v>
+      </x:c>
+      <x:c r="J430" s="6" t="str"/>
+      <x:c r="K430" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank02_roche_annual-report-2025.pdf</x:v>
+      </x:c>
+      <x:c r="L430" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M430" s="6" t="str">
+        <x:v>roche.com</x:v>
+      </x:c>
+      <x:c r="N430" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O430" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/official_snapshots/rank02_roche_annual-report-2025.html</x:v>
+      </x:c>
+      <x:c r="P430" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="431">
+      <x:c r="A431" s="6" t="str">
+        <x:v>peerpdf-0003</x:v>
+      </x:c>
+      <x:c r="B431" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C431" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D431" s="6" t="str">
+        <x:v>Pfizer 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E431" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F431" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G431" s="6" t="str"/>
+      <x:c r="H431" s="6" t="str"/>
+      <x:c r="I431" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=78003</x:v>
+      </x:c>
+      <x:c r="J431" s="6" t="str"/>
+      <x:c r="K431" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank04_pfizer_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L431" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M431" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N431" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O431" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank04_pfizer_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P431" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="432">
+      <x:c r="A432" s="6" t="str">
+        <x:v>peerpdf-0004</x:v>
+      </x:c>
+      <x:c r="B432" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C432" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D432" s="6" t="str">
+        <x:v>AbbVie 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E432" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F432" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G432" s="6" t="str"/>
+      <x:c r="H432" s="6" t="str"/>
+      <x:c r="I432" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=1551152</x:v>
+      </x:c>
+      <x:c r="J432" s="6" t="str"/>
+      <x:c r="K432" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank05_abbvie_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L432" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M432" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N432" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O432" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank05_abbvie_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P432" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="433">
+      <x:c r="A433" s="6" t="str">
+        <x:v>peerpdf-0005</x:v>
+      </x:c>
+      <x:c r="B433" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C433" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D433" s="6" t="str">
+        <x:v>AstraZeneca 2025 20-F annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E433" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F433" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G433" s="6" t="str"/>
+      <x:c r="H433" s="6" t="str"/>
+      <x:c r="I433" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=901832</x:v>
+      </x:c>
+      <x:c r="J433" s="6" t="str"/>
+      <x:c r="K433" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank06_astrazeneca_20-f_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L433" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M433" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N433" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O433" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank06_astrazeneca_20-f_2025.html</x:v>
+      </x:c>
+      <x:c r="P433" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="434">
+      <x:c r="A434" s="6" t="str">
+        <x:v>peerpdf-0006</x:v>
+      </x:c>
+      <x:c r="B434" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C434" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D434" s="6" t="str">
+        <x:v>Novartis 2025 20-F annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E434" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F434" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G434" s="6" t="str"/>
+      <x:c r="H434" s="6" t="str"/>
+      <x:c r="I434" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=1114448</x:v>
+      </x:c>
+      <x:c r="J434" s="6" t="str"/>
+      <x:c r="K434" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank07_novartis_20-f_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L434" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M434" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N434" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O434" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank07_novartis_20-f_2025.html</x:v>
+      </x:c>
+      <x:c r="P434" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="435">
+      <x:c r="A435" s="6" t="str">
+        <x:v>peerpdf-0007</x:v>
+      </x:c>
+      <x:c r="B435" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C435" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D435" s="6" t="str">
+        <x:v>Bristol Myers Squibb 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E435" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F435" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G435" s="6" t="str"/>
+      <x:c r="H435" s="6" t="str"/>
+      <x:c r="I435" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=14272</x:v>
+      </x:c>
+      <x:c r="J435" s="6" t="str"/>
+      <x:c r="K435" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank08_bristol-myers-squibb_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L435" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M435" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N435" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O435" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank08_bristol-myers-squibb_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P435" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="436">
+      <x:c r="A436" s="6" t="str">
+        <x:v>peerpdf-0008</x:v>
+      </x:c>
+      <x:c r="B436" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C436" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D436" s="6" t="str">
+        <x:v>Eli Lilly 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E436" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F436" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G436" s="6" t="str"/>
+      <x:c r="H436" s="6" t="str"/>
+      <x:c r="I436" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=59478</x:v>
+      </x:c>
+      <x:c r="J436" s="6" t="str"/>
+      <x:c r="K436" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank09_eli-lilly_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L436" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M436" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N436" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O436" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank09_eli-lilly_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P436" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="437">
+      <x:c r="A437" s="6" t="str">
+        <x:v>peerpdf-0009</x:v>
+      </x:c>
+      <x:c r="B437" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C437" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D437" s="6" t="str">
+        <x:v>Sanofi 2025 20-F annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E437" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F437" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G437" s="6" t="str"/>
+      <x:c r="H437" s="6" t="str"/>
+      <x:c r="I437" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=1121404</x:v>
+      </x:c>
+      <x:c r="J437" s="6" t="str"/>
+      <x:c r="K437" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank10_sanofi_20-f_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L437" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M437" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N437" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O437" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank10_sanofi_20-f_2025.html</x:v>
+      </x:c>
+      <x:c r="P437" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="438">
+      <x:c r="A438" s="6" t="str">
+        <x:v>peerpdf-0010</x:v>
+      </x:c>
+      <x:c r="B438" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C438" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D438" s="6" t="str">
+        <x:v>Novo Nordisk 2025 20-F annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E438" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F438" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G438" s="6" t="str"/>
+      <x:c r="H438" s="6" t="str"/>
+      <x:c r="I438" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=353278</x:v>
+      </x:c>
+      <x:c r="J438" s="6" t="str"/>
+      <x:c r="K438" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank11_novo-nordisk_20-f_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L438" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M438" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N438" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O438" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank11_novo-nordisk_20-f_2025.html</x:v>
+      </x:c>
+      <x:c r="P438" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="439">
+      <x:c r="A439" s="6" t="str">
+        <x:v>peerpdf-0011</x:v>
+      </x:c>
+      <x:c r="B439" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C439" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D439" s="6" t="str">
+        <x:v>GSK 2025 20-F annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E439" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F439" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G439" s="6" t="str"/>
+      <x:c r="H439" s="6" t="str"/>
+      <x:c r="I439" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=1131399</x:v>
+      </x:c>
+      <x:c r="J439" s="6" t="str"/>
+      <x:c r="K439" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank12_gsk_20-f_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L439" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M439" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N439" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O439" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank12_gsk_20-f_2025.html</x:v>
+      </x:c>
+      <x:c r="P439" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="440">
+      <x:c r="A440" s="6" t="str">
+        <x:v>peerpdf-0012</x:v>
+      </x:c>
+      <x:c r="B440" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C440" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D440" s="6" t="str">
+        <x:v>Amgen 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E440" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F440" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G440" s="6" t="str"/>
+      <x:c r="H440" s="6" t="str"/>
+      <x:c r="I440" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=318154</x:v>
+      </x:c>
+      <x:c r="J440" s="6" t="str"/>
+      <x:c r="K440" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank13_amgen_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L440" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M440" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N440" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O440" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank13_amgen_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P440" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="441">
+      <x:c r="A441" s="6" t="str">
+        <x:v>peerpdf-0013</x:v>
+      </x:c>
+      <x:c r="B441" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C441" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D441" s="6" t="str">
+        <x:v>Takeda 2025 20-F annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E441" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F441" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G441" s="6" t="str"/>
+      <x:c r="H441" s="6" t="str"/>
+      <x:c r="I441" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=1395064</x:v>
+      </x:c>
+      <x:c r="J441" s="6" t="str"/>
+      <x:c r="K441" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank14_takeda_20-f_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L441" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M441" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N441" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O441" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank14_takeda_20-f_2025.html</x:v>
+      </x:c>
+      <x:c r="P441" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="442">
+      <x:c r="A442" s="6" t="str">
+        <x:v>peerpdf-0014</x:v>
+      </x:c>
+      <x:c r="B442" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C442" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D442" s="6" t="str">
+        <x:v>Gilead Sciences 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E442" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F442" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G442" s="6" t="str"/>
+      <x:c r="H442" s="6" t="str"/>
+      <x:c r="I442" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=882095</x:v>
+      </x:c>
+      <x:c r="J442" s="6" t="str"/>
+      <x:c r="K442" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank16_gilead-sciences_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L442" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M442" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N442" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O442" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank16_gilead-sciences_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P442" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="443">
+      <x:c r="A443" s="6" t="str">
+        <x:v>peerpdf-0015</x:v>
+      </x:c>
+      <x:c r="B443" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C443" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D443" s="6" t="str">
+        <x:v>Merck KGaA / EMD Group Annual Report 2025 PDF export</x:v>
+      </x:c>
+      <x:c r="E443" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F443" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G443" s="6" t="str"/>
+      <x:c r="H443" s="6" t="str"/>
+      <x:c r="I443" s="6" t="str">
+        <x:v>https://reports.emdgroup.com/en/annualreport/2025/</x:v>
+      </x:c>
+      <x:c r="J443" s="6" t="str"/>
+      <x:c r="K443" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank18_merck-kgaa-emd-group_annual-report-2025.pdf</x:v>
+      </x:c>
+      <x:c r="L443" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M443" s="6" t="str">
+        <x:v>reports.emdgroup.com</x:v>
+      </x:c>
+      <x:c r="N443" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O443" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/official_snapshots/rank18_merck-kgaa-emd-group_annual-report-2025.html</x:v>
+      </x:c>
+      <x:c r="P443" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="444">
+      <x:c r="A444" s="6" t="str">
+        <x:v>peerpdf-0016</x:v>
+      </x:c>
+      <x:c r="B444" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C444" s="6" t="str">
+        <x:v>pdf_exports</x:v>
+      </x:c>
+      <x:c r="D444" s="6" t="str">
+        <x:v>Teva Pharmaceutical 2025 10-K annual report PDF export</x:v>
+      </x:c>
+      <x:c r="E444" s="6" t="str">
+        <x:v>peer_annual_report_pdf_export</x:v>
+      </x:c>
+      <x:c r="F444" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G444" s="6" t="str"/>
+      <x:c r="H444" s="6" t="str"/>
+      <x:c r="I444" s="6" t="str">
+        <x:v>https://www.sec.gov/edgar/browse/?CIK=818686</x:v>
+      </x:c>
+      <x:c r="J444" s="6" t="str"/>
+      <x:c r="K444" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank19_teva-pharmaceutical_10-k_2025.pdf</x:v>
+      </x:c>
+      <x:c r="L444" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M444" s="6" t="str">
+        <x:v>sec.gov</x:v>
+      </x:c>
+      <x:c r="N444" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O444" s="6" t="str">
+        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/sec_filings/rank19_teva-pharmaceutical_10-k_2025.html</x:v>
+      </x:c>
+      <x:c r="P444" s="6" t="str">
+        <x:v>generated</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="P2:P428">
+  <x:conditionalFormatting sqref="P2:P444">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="failed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="metadata_only"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="duplicate"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0d5225869734fcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R872020a49d254c1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Replace Roche peer export with official PDF
</commit_message>
<xml_diff>
--- a/Merck Official Hackathon Corpus/manifest.xlsx
+++ b/Merck Official Hackathon Corpus/manifest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R884b4b3bcbdb44b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R4f7b3acd805b4ab4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20274,44 +20274,44 @@
         <x:v>07_peer_pharma_annual_reports</x:v>
       </x:c>
       <x:c r="C411" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/official_snapshots</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports</x:v>
       </x:c>
       <x:c r="D411" s="6" t="str">
         <x:v>Roche Annual Report 2025</x:v>
       </x:c>
       <x:c r="E411" s="6" t="str">
-        <x:v>peer_annual_report_official_snapshot</x:v>
+        <x:v>peer_annual_report_official_pdf</x:v>
       </x:c>
       <x:c r="F411" s="6" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="G411" s="6" t="str"/>
       <x:c r="H411" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2025-01-29</x:v>
       </x:c>
       <x:c r="I411" s="6" t="str">
         <x:v>https://www.roche.com/investors/annualreport25</x:v>
       </x:c>
       <x:c r="J411" s="6" t="str">
-        <x:v>https://www.roche.com/investors/annualreport25</x:v>
+        <x:v>https://assets.roche.com/f/176343/x/fa3c863601/ar25e.pdf</x:v>
       </x:c>
       <x:c r="K411" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/official_snapshots/rank02_roche_annual-report-2025.html</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports/rank02_roche_annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="L411" s="6" t="str">
-        <x:v>html</x:v>
+        <x:v>pdf</x:v>
       </x:c>
       <x:c r="M411" s="6" t="str">
-        <x:v>www.roche.com</x:v>
+        <x:v>assets.roche.com</x:v>
       </x:c>
       <x:c r="N411" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O411" s="6" t="str">
-        <x:v>Top-20 pharma rank 2; 2024 pharma revenue 65.3B. Official Roche Annual Report 2025 page snapshot. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
+        <x:v>Top-20 pharma rank 2; 2024 pharma revenue 65.3B. Official Roche Annual Report 2025 English PDF downloaded from Roche assets. HTML landing-page snapshot retained at 07_peer_pharma_annual_reports/official_snapshots/rank02_roche_annual-report-2025.html.</x:v>
       </x:c>
       <x:c r="P411" s="6" t="str">
-        <x:v>snapshot_saved</x:v>
+        <x:v>downloaded</x:v>
       </x:c>
     </x:row>
     <x:row r="412">
@@ -21181,10 +21181,10 @@
         <x:v>pdf_exports</x:v>
       </x:c>
       <x:c r="D430" s="6" t="str">
-        <x:v>Roche Annual Report 2025 PDF export</x:v>
+        <x:v>Roche Annual Report 2025 English PDF</x:v>
       </x:c>
       <x:c r="E430" s="6" t="str">
-        <x:v>peer_annual_report_pdf_export</x:v>
+        <x:v>peer_annual_report_official_pdf</x:v>
       </x:c>
       <x:c r="F430" s="6" t="str">
         <x:v>2025</x:v>
@@ -21192,7 +21192,7 @@
       <x:c r="G430" s="6" t="str"/>
       <x:c r="H430" s="6" t="str"/>
       <x:c r="I430" s="6" t="str">
-        <x:v>https://www.roche.com/investors/annualreport25</x:v>
+        <x:v>https://assets.roche.com/f/176343/x/fa3c863601/ar25e.pdf</x:v>
       </x:c>
       <x:c r="J430" s="6" t="str"/>
       <x:c r="K430" s="6" t="str">
@@ -21202,16 +21202,16 @@
         <x:v>pdf</x:v>
       </x:c>
       <x:c r="M430" s="6" t="str">
-        <x:v>roche.com</x:v>
+        <x:v>assets.roche.com</x:v>
       </x:c>
       <x:c r="N430" s="6" t="str">
         <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O430" s="6" t="str">
-        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/official_snapshots/rank02_roche_annual-report-2025.html</x:v>
+        <x:v>Official Roche Annual Report 2025 English PDF copied into pdf_exports after the generated landing-page PDF was found to be incomplete.</x:v>
       </x:c>
       <x:c r="P430" s="6" t="str">
-        <x:v>generated</x:v>
+        <x:v>downloaded</x:v>
       </x:c>
     </x:row>
     <x:row r="431">
@@ -21838,7 +21838,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R872020a49d254c1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1962860ef3384fa1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Replace Merck KGaA peer export with official PDF
</commit_message>
<xml_diff>
--- a/Merck Official Hackathon Corpus/manifest.xlsx
+++ b/Merck Official Hackathon Corpus/manifest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R4f7b3acd805b4ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="Rc9ed18cd802f4d18"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20990,44 +20990,44 @@
         <x:v>07_peer_pharma_annual_reports</x:v>
       </x:c>
       <x:c r="C426" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/official_snapshots</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports</x:v>
       </x:c>
       <x:c r="D426" s="6" t="str">
         <x:v>Merck KGaA / EMD Group Annual Report 2025</x:v>
       </x:c>
       <x:c r="E426" s="6" t="str">
-        <x:v>peer_annual_report_official_snapshot</x:v>
+        <x:v>peer_annual_report_official_pdf</x:v>
       </x:c>
       <x:c r="F426" s="6" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="G426" s="6" t="str"/>
       <x:c r="H426" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-03-05</x:v>
       </x:c>
       <x:c r="I426" s="6" t="str">
         <x:v>https://reports.emdgroup.com/en/annualreport/2025/</x:v>
       </x:c>
       <x:c r="J426" s="6" t="str">
-        <x:v>https://reports.emdgroup.com/en/annualreport/2025/</x:v>
+        <x:v>https://reports.emdgroup.com/en/annualreport/2025/_assets/downloads/entire-emd-ar25.pdf</x:v>
       </x:c>
       <x:c r="K426" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/official_snapshots/rank18_merck-kgaa-emd-group_annual-report-2025.html</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports/rank18_merck-kgaa-emd-group_annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="L426" s="6" t="str">
-        <x:v>html</x:v>
+        <x:v>pdf</x:v>
       </x:c>
       <x:c r="M426" s="6" t="str">
         <x:v>reports.emdgroup.com</x:v>
       </x:c>
       <x:c r="N426" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O426" s="6" t="str">
-        <x:v>Top-20 pharma rank 18; 2024 pharma revenue 19.1B. Official Merck KGaA / EMD Group Annual Report 2025 page snapshot. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
+        <x:v>Top-20 pharma rank 18; 2024 pharma revenue 19.1B. Official Annual Report 2025 PDF downloaded from Merck KGaA / EMD Group downloads page. HTML landing-page snapshot retained at 07_peer_pharma_annual_reports/official_snapshots/rank18_merck-kgaa-emd-group_annual-report-2025.html.</x:v>
       </x:c>
       <x:c r="P426" s="6" t="str">
-        <x:v>snapshot_saved</x:v>
+        <x:v>downloaded</x:v>
       </x:c>
     </x:row>
     <x:row r="427">
@@ -21099,28 +21099,28 @@
       </x:c>
       <x:c r="G428" s="6" t="str"/>
       <x:c r="H428" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-03-05</x:v>
       </x:c>
       <x:c r="I428" s="6" t="str">
         <x:v>https://www.csl.com/-/media/shared/documents/annual-report/csl-annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="J428" s="6" t="str">
-        <x:v>https://www.csl.com/-/media/shared/documents/annual-report/csl-annual-report-2025.pdf</x:v>
+        <x:v>https://reports.emdgroup.com/en/annualreport/2025/_assets/downloads/entire-emd-ar25.pdf</x:v>
       </x:c>
       <x:c r="K428" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/official_reports/rank20_csl_annual-report-2025.pdf</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports/rank18_merck-kgaa-emd-group_annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="L428" s="6" t="str">
         <x:v>pdf</x:v>
       </x:c>
       <x:c r="M428" s="6" t="str">
-        <x:v>www.csl.com</x:v>
+        <x:v>reports.emdgroup.com</x:v>
       </x:c>
       <x:c r="N428" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O428" s="6" t="str">
-        <x:v>Top-20 pharma rank 20; 2024 pharma revenue 15.2B. Official CSL Annual Report 2025 PDF from CSL investor annual reports page. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
+        <x:v>Top-20 pharma rank 18; 2024 pharma revenue 19.1B. Official Annual Report 2025 PDF downloaded from Merck KGaA / EMD Group downloads page. HTML landing-page snapshot retained at 07_peer_pharma_annual_reports/official_snapshots/rank18_merck-kgaa-emd-group_annual-report-2025.html.</x:v>
       </x:c>
       <x:c r="P428" s="6" t="str">
         <x:v>downloaded</x:v>
@@ -21753,10 +21753,10 @@
         <x:v>pdf_exports</x:v>
       </x:c>
       <x:c r="D443" s="6" t="str">
-        <x:v>Merck KGaA / EMD Group Annual Report 2025 PDF export</x:v>
+        <x:v>Merck KGaA / EMD Group Annual Report 2025 PDF</x:v>
       </x:c>
       <x:c r="E443" s="6" t="str">
-        <x:v>peer_annual_report_pdf_export</x:v>
+        <x:v>peer_annual_report_official_pdf</x:v>
       </x:c>
       <x:c r="F443" s="6" t="str">
         <x:v>2025</x:v>
@@ -21764,7 +21764,7 @@
       <x:c r="G443" s="6" t="str"/>
       <x:c r="H443" s="6" t="str"/>
       <x:c r="I443" s="6" t="str">
-        <x:v>https://reports.emdgroup.com/en/annualreport/2025/</x:v>
+        <x:v>https://reports.emdgroup.com/en/annualreport/2025/_assets/downloads/entire-emd-ar25.pdf</x:v>
       </x:c>
       <x:c r="J443" s="6" t="str"/>
       <x:c r="K443" s="6" t="str">
@@ -21780,10 +21780,10 @@
         <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O443" s="6" t="str">
-        <x:v>Generated from locally saved official HTML filing/snapshot for easier LLM upload and review. Source HTML: 07_peer_pharma_annual_reports/official_snapshots/rank18_merck-kgaa-emd-group_annual-report-2025.html</x:v>
+        <x:v>Official Merck KGaA / EMD Group Annual Report 2025 PDF copied into pdf_exports after the generated landing-page PDF was found to be incomplete.</x:v>
       </x:c>
       <x:c r="P443" s="6" t="str">
-        <x:v>generated</x:v>
+        <x:v>downloaded</x:v>
       </x:c>
     </x:row>
     <x:row r="444">
@@ -21838,7 +21838,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1962860ef3384fa1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0df76ed19df4ac9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update blocked peer pharma metadata
</commit_message>
<xml_diff>
--- a/Merck Official Hackathon Corpus/manifest.xlsx
+++ b/Merck Official Hackathon Corpus/manifest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="Rc9ed18cd802f4d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R40227630bfca44ad"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20947,7 +20947,7 @@
         <x:v>07_peer_pharma_annual_reports/metadata_only</x:v>
       </x:c>
       <x:c r="D425" s="6" t="str">
-        <x:v>Bayer Annual Reports Page</x:v>
+        <x:v>Bayer Annual Report 2025</x:v>
       </x:c>
       <x:c r="E425" s="6" t="str">
         <x:v>peer_annual_report_metadata</x:v>
@@ -20957,13 +20957,13 @@
       </x:c>
       <x:c r="G425" s="6" t="str"/>
       <x:c r="H425" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-03</x:v>
       </x:c>
       <x:c r="I425" s="6" t="str">
         <x:v>https://www.bayer.com/en/investors/annual-reports</x:v>
       </x:c>
       <x:c r="J425" s="6" t="str">
-        <x:v>https://www.bayer.com/en/investors/annual-reports</x:v>
+        <x:v>https://www.bayer.com/sites/default/files/2026-03/bayer-annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="K425" s="6" t="str"/>
       <x:c r="L425" s="6" t="str">
@@ -20973,10 +20973,10 @@
         <x:v>www.bayer.com</x:v>
       </x:c>
       <x:c r="N425" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O425" s="6" t="str">
-        <x:v>Top-20 pharma rank 17; 2024 pharma revenue 26.0B. Official annual-report page identified, but automated download was blocked by site protection. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
+        <x:v>Top-20 pharma rank 17; 2024 pharma revenue 26.0B. Official Bayer Annual Report 2025 PDF URL verified through a rendered text view, but automated binary download was blocked by Bayer site protection with HTTP 403. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
       </x:c>
       <x:c r="P425" s="6" t="str">
         <x:v>metadata_only</x:v>
@@ -21099,28 +21099,28 @@
       </x:c>
       <x:c r="G428" s="6" t="str"/>
       <x:c r="H428" s="6" t="str">
-        <x:v>2026-03-05</x:v>
+        <x:v>2026-06-12</x:v>
       </x:c>
       <x:c r="I428" s="6" t="str">
         <x:v>https://www.csl.com/-/media/shared/documents/annual-report/csl-annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="J428" s="6" t="str">
-        <x:v>https://reports.emdgroup.com/en/annualreport/2025/_assets/downloads/entire-emd-ar25.pdf</x:v>
+        <x:v>https://www.csl.com/-/media/shared/documents/annual-report/csl-annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="K428" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/official_reports/rank18_merck-kgaa-emd-group_annual-report-2025.pdf</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports/rank20_csl_annual-report-2025.pdf</x:v>
       </x:c>
       <x:c r="L428" s="6" t="str">
         <x:v>pdf</x:v>
       </x:c>
       <x:c r="M428" s="6" t="str">
-        <x:v>reports.emdgroup.com</x:v>
+        <x:v>www.csl.com</x:v>
       </x:c>
       <x:c r="N428" s="6" t="str">
-        <x:v>2026-06-24</x:v>
+        <x:v>2026-06-12</x:v>
       </x:c>
       <x:c r="O428" s="6" t="str">
-        <x:v>Top-20 pharma rank 18; 2024 pharma revenue 19.1B. Official Annual Report 2025 PDF downloaded from Merck KGaA / EMD Group downloads page. HTML landing-page snapshot retained at 07_peer_pharma_annual_reports/official_snapshots/rank18_merck-kgaa-emd-group_annual-report-2025.html.</x:v>
+        <x:v>Top-20 pharma rank 20; 2024 pharma revenue 15.2B. Official CSL Annual Report 2025 PDF from CSL investor annual reports page.</x:v>
       </x:c>
       <x:c r="P428" s="6" t="str">
         <x:v>downloaded</x:v>
@@ -21838,7 +21838,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0df76ed19df4ac9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R585f31a5b5d74800"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add manually downloaded Bayer and Boehringer reports
</commit_message>
<xml_diff>
--- a/Merck Official Hackathon Corpus/manifest.xlsx
+++ b/Merck Official Hackathon Corpus/manifest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R40227630bfca44ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manifest" sheetId="1" r:id="R501e229114b44340"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,8 +131,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifestTable" displayName="ManifestTable" ref="A1:P444" headerRowCount="1">
-  <x:autoFilter ref="A1:P444"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ManifestTable" displayName="ManifestTable" ref="A1:P446" headerRowCount="1">
+  <x:autoFilter ref="A1:P446"/>
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="repository"/>
@@ -20850,42 +20850,44 @@
         <x:v>07_peer_pharma_annual_reports</x:v>
       </x:c>
       <x:c r="C423" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/metadata_only</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports</x:v>
       </x:c>
       <x:c r="D423" s="6" t="str">
-        <x:v>Boehringer Ingelheim Annual Report 2025</x:v>
+        <x:v>Boehringer Ingelheim Annual Report Highlights 2025</x:v>
       </x:c>
       <x:c r="E423" s="6" t="str">
-        <x:v>peer_annual_report_metadata</x:v>
+        <x:v>peer_annual_report_official_pdf</x:v>
       </x:c>
       <x:c r="F423" s="6" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="G423" s="6" t="str"/>
       <x:c r="H423" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-03-19</x:v>
       </x:c>
       <x:c r="I423" s="6" t="str">
-        <x:v>https://annualreport.boehringer-ingelheim.com/2025/</x:v>
+        <x:v>https://www.boehringer-ingelheim.com/annualreport/2025/</x:v>
       </x:c>
       <x:c r="J423" s="6" t="str">
-        <x:v>https://annualreport.boehringer-ingelheim.com/2025/</x:v>
-      </x:c>
-      <x:c r="K423" s="6" t="str"/>
+        <x:v>https://www.boehringer-ingelheim.com/annualreport/2025/files/Boehringer-Ingelheim-Annual-Report-Highlights-2025.pdf</x:v>
+      </x:c>
+      <x:c r="K423" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/official_reports/rank15_boehringer-ingelheim_annual-report-highlights-2025.pdf</x:v>
+      </x:c>
       <x:c r="L423" s="6" t="str">
-        <x:v>link</x:v>
+        <x:v>pdf</x:v>
       </x:c>
       <x:c r="M423" s="6" t="str">
-        <x:v>annualreport.boehringer-ingelheim.com</x:v>
+        <x:v>www.boehringer-ingelheim.com</x:v>
       </x:c>
       <x:c r="N423" s="6" t="str">
-        <x:v>2026-06-12</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O423" s="6" t="str">
-        <x:v>Top-20 pharma rank 15; 2024 pharma revenue 29.0B. Official annual-report page identified, but automated download was blocked by site protection. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
+        <x:v>Top-20 pharma rank 15; 2024 pharma revenue 29.0B. Official 38-page Annual Report 2025 Highlights PDF manually downloaded from Boehringer Ingelheim official annual-report site. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
       </x:c>
       <x:c r="P423" s="6" t="str">
-        <x:v>metadata_only</x:v>
+        <x:v>downloaded</x:v>
       </x:c>
     </x:row>
     <x:row r="424">
@@ -20944,20 +20946,20 @@
         <x:v>07_peer_pharma_annual_reports</x:v>
       </x:c>
       <x:c r="C425" s="6" t="str">
-        <x:v>07_peer_pharma_annual_reports/metadata_only</x:v>
+        <x:v>07_peer_pharma_annual_reports/official_reports</x:v>
       </x:c>
       <x:c r="D425" s="6" t="str">
         <x:v>Bayer Annual Report 2025</x:v>
       </x:c>
       <x:c r="E425" s="6" t="str">
-        <x:v>peer_annual_report_metadata</x:v>
+        <x:v>peer_annual_report_official_pdf</x:v>
       </x:c>
       <x:c r="F425" s="6" t="str">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="G425" s="6" t="str"/>
       <x:c r="H425" s="6" t="str">
-        <x:v>2026-03</x:v>
+        <x:v>2026-03-05</x:v>
       </x:c>
       <x:c r="I425" s="6" t="str">
         <x:v>https://www.bayer.com/en/investors/annual-reports</x:v>
@@ -20965,9 +20967,11 @@
       <x:c r="J425" s="6" t="str">
         <x:v>https://www.bayer.com/sites/default/files/2026-03/bayer-annual-report-2025.pdf</x:v>
       </x:c>
-      <x:c r="K425" s="6" t="str"/>
+      <x:c r="K425" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/official_reports/rank17_bayer_annual-report-2025.pdf</x:v>
+      </x:c>
       <x:c r="L425" s="6" t="str">
-        <x:v>link</x:v>
+        <x:v>pdf</x:v>
       </x:c>
       <x:c r="M425" s="6" t="str">
         <x:v>www.bayer.com</x:v>
@@ -20976,10 +20980,10 @@
         <x:v>2026-06-24</x:v>
       </x:c>
       <x:c r="O425" s="6" t="str">
-        <x:v>Top-20 pharma rank 17; 2024 pharma revenue 26.0B. Official Bayer Annual Report 2025 PDF URL verified through a rendered text view, but automated binary download was blocked by Bayer site protection with HTTP 403. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
+        <x:v>Top-20 pharma rank 17; 2024 pharma revenue 26.0B. Official Bayer Annual Report 2025 PDF manually downloaded from Bayer official annual-report site after automated binary download was blocked. Ranking source: https://en.wikipedia.org/wiki/Pharmaceutical_industry#Global_sales</x:v>
       </x:c>
       <x:c r="P425" s="6" t="str">
-        <x:v>metadata_only</x:v>
+        <x:v>downloaded</x:v>
       </x:c>
     </x:row>
     <x:row r="426">
@@ -21830,15 +21834,111 @@
         <x:v>generated</x:v>
       </x:c>
     </x:row>
+    <x:row r="445">
+      <x:c r="A445" s="6" t="str">
+        <x:v>peerpdf-0017</x:v>
+      </x:c>
+      <x:c r="B445" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C445" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports</x:v>
+      </x:c>
+      <x:c r="D445" s="6" t="str">
+        <x:v>Boehringer Ingelheim Annual Report Highlights 2025 PDF</x:v>
+      </x:c>
+      <x:c r="E445" s="6" t="str">
+        <x:v>peer_annual_report_official_pdf</x:v>
+      </x:c>
+      <x:c r="F445" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G445" s="6" t="str"/>
+      <x:c r="H445" s="6" t="str">
+        <x:v>2026-03-19</x:v>
+      </x:c>
+      <x:c r="I445" s="6" t="str">
+        <x:v>https://www.boehringer-ingelheim.com/annualreport/2025/</x:v>
+      </x:c>
+      <x:c r="J445" s="6" t="str">
+        <x:v>https://www.boehringer-ingelheim.com/annualreport/2025/files/Boehringer-Ingelheim-Annual-Report-Highlights-2025.pdf</x:v>
+      </x:c>
+      <x:c r="K445" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank15_boehringer-ingelheim_annual-report-highlights-2025.pdf</x:v>
+      </x:c>
+      <x:c r="L445" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M445" s="6" t="str">
+        <x:v>www.boehringer-ingelheim.com</x:v>
+      </x:c>
+      <x:c r="N445" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O445" s="6" t="str">
+        <x:v>Official peer-company PDF copied into pdf_exports for easier LLM upload and review.</x:v>
+      </x:c>
+      <x:c r="P445" s="6" t="str">
+        <x:v>downloaded</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="446">
+      <x:c r="A446" s="6" t="str">
+        <x:v>peerpdf-0018</x:v>
+      </x:c>
+      <x:c r="B446" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports</x:v>
+      </x:c>
+      <x:c r="C446" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports</x:v>
+      </x:c>
+      <x:c r="D446" s="6" t="str">
+        <x:v>Bayer Annual Report 2025 PDF</x:v>
+      </x:c>
+      <x:c r="E446" s="6" t="str">
+        <x:v>peer_annual_report_official_pdf</x:v>
+      </x:c>
+      <x:c r="F446" s="6" t="str">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G446" s="6" t="str"/>
+      <x:c r="H446" s="6" t="str">
+        <x:v>2026-03-05</x:v>
+      </x:c>
+      <x:c r="I446" s="6" t="str">
+        <x:v>https://www.bayer.com/en/investors/annual-reports</x:v>
+      </x:c>
+      <x:c r="J446" s="6" t="str">
+        <x:v>https://www.bayer.com/sites/default/files/2026-03/bayer-annual-report-2025.pdf</x:v>
+      </x:c>
+      <x:c r="K446" s="6" t="str">
+        <x:v>07_peer_pharma_annual_reports/pdf_exports/rank17_bayer_annual-report-2025.pdf</x:v>
+      </x:c>
+      <x:c r="L446" s="6" t="str">
+        <x:v>pdf</x:v>
+      </x:c>
+      <x:c r="M446" s="6" t="str">
+        <x:v>www.bayer.com</x:v>
+      </x:c>
+      <x:c r="N446" s="6" t="str">
+        <x:v>2026-06-24</x:v>
+      </x:c>
+      <x:c r="O446" s="6" t="str">
+        <x:v>Official peer-company PDF copied into pdf_exports for easier LLM upload and review.</x:v>
+      </x:c>
+      <x:c r="P446" s="6" t="str">
+        <x:v>downloaded</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="P2:P444">
+  <x:conditionalFormatting sqref="P2:P446">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="failed"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="metadata_only"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="duplicate"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R585f31a5b5d74800"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb15f64526a44b4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>